<commit_message>
Informe del Sprint 1 en PDF y estado del sprint actualizado
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01. Inicio/Backlog del Producto.xlsx
+++ b/01. Inicio/Backlog del Producto.xlsx
@@ -1526,12 +1526,12 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">En Progreso</t>
+          <t xml:space="preserve">Terminado</t>
         </is>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Acta lista; falta firmarla. Fase CRISP-ML(Q): comprensión del negocio y de los datos</t>
+          <t xml:space="preserve">Acta firmada. Fase CRISP-ML(Q): comprensión del negocio y de los datos</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por Hacer</t>
+          <t xml:space="preserve">Terminado</t>
         </is>
       </c>
       <c r="P9" s="9" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por Hacer</t>
+          <t xml:space="preserve">Terminado</t>
         </is>
       </c>
       <c r="P10" s="9" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por Hacer</t>
+          <t xml:space="preserve">Terminado</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">

</xml_diff>